<commit_message>
ParcelPilot AI Agent - Assessment Submission
</commit_message>
<xml_diff>
--- a/data/excel/ParcelPilot_Assessment_Data.xlsx
+++ b/data/excel/ParcelPilot_Assessment_Data.xlsx
@@ -1,15 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\chatbot ai agent\data\excel\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B4E789D-B903-4812-973B-E2D3E441D6A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="README" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="accounts" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="orders" sheetId="3" r:id="rId7"/>
-    <sheet state="visible" name="tickets" sheetId="4" r:id="rId8"/>
+    <sheet name="README" sheetId="1" r:id="rId1"/>
+    <sheet name="accounts" sheetId="2" r:id="rId2"/>
+    <sheet name="orders" sheetId="3" r:id="rId3"/>
+    <sheet name="tickets" sheetId="4" r:id="rId4"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -421,28 +430,28 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4">
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Carlito"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Carlito"/>
     </font>
     <font>
       <b/>
-      <sz val="16.0"/>
+      <sz val="16"/>
       <color theme="1"/>
       <name val="Carlito"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Carlito"/>
     </font>
@@ -452,58 +461,52 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -693,55 +696,56 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B1000"/>
+  <sheetFormatPr defaultColWidth="12.59765625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="55.63"/>
-    <col customWidth="1" min="2" max="2" width="55.0"/>
-    <col customWidth="1" min="3" max="26" width="8.63"/>
+    <col min="1" max="1" width="55.59765625" customWidth="1"/>
+    <col min="2" max="2" width="55" customWidth="1"/>
+    <col min="3" max="26" width="8.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:2" ht="15.6">
+      <c r="A1" s="3" t="s">
         <v>2</v>
       </c>
+      <c r="B1" s="4"/>
     </row>
-    <row r="2">
+    <row r="2" spans="1:2" ht="13.8">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:2" ht="13.8">
       <c r="A3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:2" ht="13.8">
       <c r="A4" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:2" ht="27.6">
       <c r="A5" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>30</v>
       </c>
     </row>
@@ -1729,32 +1733,28 @@
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>
   </mergeCells>
-  <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:H1000"/>
+  <sheetFormatPr defaultColWidth="12.59765625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="8.88"/>
-    <col customWidth="1" min="2" max="2" width="14.38"/>
-    <col customWidth="1" min="3" max="3" width="8.25"/>
-    <col customWidth="1" min="4" max="4" width="5.13"/>
-    <col customWidth="1" min="5" max="5" width="10.25"/>
-    <col customWidth="1" min="6" max="6" width="35.0"/>
-    <col customWidth="1" min="7" max="7" width="14.38"/>
-    <col customWidth="1" min="8" max="8" width="35.0"/>
-    <col customWidth="1" min="9" max="26" width="8.63"/>
+    <col min="1" max="1" width="8.8984375" customWidth="1"/>
+    <col min="2" max="2" width="14.3984375" customWidth="1"/>
+    <col min="3" max="3" width="8.19921875" customWidth="1"/>
+    <col min="4" max="4" width="5.09765625" customWidth="1"/>
+    <col min="5" max="5" width="10.19921875" customWidth="1"/>
+    <col min="6" max="6" width="35" customWidth="1"/>
+    <col min="7" max="7" width="14.3984375" customWidth="1"/>
+    <col min="8" max="8" width="35" customWidth="1"/>
+    <col min="9" max="26" width="8.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:8" ht="27.6">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -1780,103 +1780,103 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:8" ht="27.6">
+      <c r="A2" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="G2" s="3" t="b">
+      <c r="G2" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="2" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:8" ht="27.6">
+      <c r="A3" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="G3" s="3" t="b">
+      <c r="G3" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="2" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:8" ht="27.6">
+      <c r="A4" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3" t="b">
+      <c r="F4" s="2"/>
+      <c r="G4" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="2" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:8" ht="27.6">
+      <c r="A5" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3" t="b">
+      <c r="F5" s="2"/>
+      <c r="G5" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="H5" s="2" t="s">
         <v>98</v>
       </c>
     </row>
@@ -2861,37 +2861,33 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:M1000"/>
+  <sheetFormatPr defaultColWidth="12.59765625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="8.13"/>
-    <col customWidth="1" min="2" max="2" width="8.88"/>
-    <col customWidth="1" min="3" max="3" width="10.0"/>
-    <col customWidth="1" min="4" max="4" width="9.0"/>
-    <col customWidth="1" min="5" max="5" width="13.75"/>
-    <col customWidth="1" min="6" max="6" width="35.0"/>
-    <col customWidth="1" min="7" max="7" width="16.38"/>
-    <col customWidth="1" min="8" max="8" width="35.0"/>
-    <col customWidth="1" min="9" max="9" width="14.0"/>
-    <col customWidth="1" min="10" max="10" width="35.0"/>
-    <col customWidth="1" min="11" max="11" width="12.13"/>
-    <col customWidth="1" min="12" max="12" width="20.75"/>
-    <col customWidth="1" min="13" max="13" width="35.0"/>
-    <col customWidth="1" min="14" max="26" width="8.63"/>
+    <col min="1" max="1" width="8.09765625" customWidth="1"/>
+    <col min="2" max="2" width="8.8984375" customWidth="1"/>
+    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="4" max="4" width="9" customWidth="1"/>
+    <col min="5" max="5" width="13.69921875" customWidth="1"/>
+    <col min="6" max="6" width="35" customWidth="1"/>
+    <col min="7" max="7" width="16.3984375" customWidth="1"/>
+    <col min="8" max="8" width="35" customWidth="1"/>
+    <col min="9" max="9" width="14" customWidth="1"/>
+    <col min="10" max="10" width="35" customWidth="1"/>
+    <col min="11" max="11" width="12.09765625" customWidth="1"/>
+    <col min="12" max="12" width="20.69921875" customWidth="1"/>
+    <col min="13" max="13" width="35" customWidth="1"/>
+    <col min="14" max="26" width="8.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:13" ht="27.6">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -2932,239 +2928,254 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:13" ht="27.6">
+      <c r="A2" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3">
-        <v>4200.0</v>
-      </c>
-      <c r="J2" s="3" t="b">
+      <c r="H2" s="2"/>
+      <c r="I2" s="2">
+        <v>4200</v>
+      </c>
+      <c r="J2" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="K2" s="3" t="b">
+      <c r="K2" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="L2" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="M2" s="2" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:13" ht="27.6">
+      <c r="A3" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="I3" s="3">
-        <v>5100.0</v>
-      </c>
-      <c r="J3" s="3" t="b">
+      <c r="I3" s="2">
+        <v>5100</v>
+      </c>
+      <c r="J3" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="K3" s="3" t="b">
+      <c r="K3" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="L3" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="M3" s="3" t="s">
+      <c r="M3" s="2" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:13" ht="27.6">
+      <c r="A4" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3">
-        <v>1800.0</v>
-      </c>
-      <c r="J4" s="3" t="b">
+      <c r="H4" s="2"/>
+      <c r="I4" s="2">
+        <v>1800</v>
+      </c>
+      <c r="J4" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="K4" s="3" t="b">
+      <c r="K4" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="L4" s="3" t="s">
+      <c r="L4" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="M4" s="3" t="s">
+      <c r="M4" s="2" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:13" ht="27.6">
+      <c r="A5" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3">
-        <v>2400.0</v>
-      </c>
-      <c r="J5" s="3" t="b">
+      <c r="H5" s="2"/>
+      <c r="I5" s="2">
+        <v>2400</v>
+      </c>
+      <c r="J5" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="K5" s="3" t="b">
+      <c r="K5" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="L5" s="3"/>
-      <c r="M5" s="3" t="s">
+      <c r="L5" s="2"/>
+      <c r="M5" s="2" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="s">
+    <row r="6" spans="1:13" ht="27.6">
+      <c r="A6" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G6" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3">
-        <v>1200.0</v>
-      </c>
-      <c r="J6" s="3" t="b">
+      <c r="H6" s="2"/>
+      <c r="I6" s="2">
+        <v>1200</v>
+      </c>
+      <c r="J6" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="K6" s="3" t="b">
+      <c r="K6" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="L6" s="3" t="s">
+      <c r="L6" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="M6" s="3" t="s">
+      <c r="M6" s="2" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="3" t="s">
+    <row r="7" spans="1:13" ht="27.6">
+      <c r="A7" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="G7" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="H7" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="I7" s="3">
-        <v>3600.0</v>
-      </c>
-      <c r="J7" s="3" t="b">
+      <c r="I7" s="2">
+        <v>3600</v>
+      </c>
+      <c r="J7" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="K7" s="3" t="b">
+      <c r="K7" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="L7" s="3"/>
-      <c r="M7" s="3" t="s">
+      <c r="L7" s="2"/>
+      <c r="M7" s="2" t="s">
         <v>133</v>
       </c>
+    </row>
+    <row r="8" spans="1:13" ht="15" customHeight="1">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
+      <c r="L8" s="2"/>
+      <c r="M8" s="2"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -4147,34 +4158,30 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:J1000"/>
+  <sheetFormatPr defaultColWidth="12.59765625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="7.13"/>
-    <col customWidth="1" min="2" max="2" width="8.88"/>
-    <col customWidth="1" min="3" max="3" width="13.75"/>
-    <col customWidth="1" min="4" max="4" width="5.38"/>
-    <col customWidth="1" min="5" max="5" width="40.88"/>
-    <col customWidth="1" min="6" max="6" width="35.0"/>
-    <col customWidth="1" min="7" max="7" width="6.5"/>
-    <col customWidth="1" min="8" max="8" width="35.0"/>
-    <col customWidth="1" min="9" max="9" width="21.25"/>
-    <col customWidth="1" min="10" max="10" width="35.0"/>
-    <col customWidth="1" min="11" max="26" width="8.63"/>
+    <col min="1" max="1" width="7.09765625" customWidth="1"/>
+    <col min="2" max="2" width="8.8984375" customWidth="1"/>
+    <col min="3" max="3" width="13.69921875" customWidth="1"/>
+    <col min="4" max="4" width="5.3984375" customWidth="1"/>
+    <col min="5" max="5" width="40.8984375" customWidth="1"/>
+    <col min="6" max="6" width="35" customWidth="1"/>
+    <col min="7" max="7" width="6.5" customWidth="1"/>
+    <col min="8" max="8" width="35" customWidth="1"/>
+    <col min="9" max="9" width="21.19921875" customWidth="1"/>
+    <col min="10" max="10" width="35" customWidth="1"/>
+    <col min="11" max="26" width="8.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:10" ht="27.6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4206,217 +4213,217 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:10" ht="41.4">
+      <c r="A2" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="J2" s="3"/>
+      <c r="J2" s="2"/>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:10" ht="41.4">
+      <c r="A3" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I3" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="J3" s="3"/>
+      <c r="J3" s="2"/>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:10" ht="27.6">
+      <c r="A4" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="J4" s="3"/>
+      <c r="J4" s="2"/>
     </row>
-    <row r="5">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:10" ht="41.4">
+      <c r="A5" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="H5" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="I5" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="J5" s="3"/>
+      <c r="J5" s="2"/>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="s">
+    <row r="6" spans="1:10" ht="55.2">
+      <c r="A6" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G6" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="H6" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="I6" s="3" t="s">
+      <c r="I6" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="J6" s="3"/>
+      <c r="J6" s="2"/>
     </row>
-    <row r="7">
-      <c r="A7" s="3" t="s">
+    <row r="7" spans="1:10" ht="41.4">
+      <c r="A7" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="G7" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="H7" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="I7" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="J7" s="3" t="s">
+      <c r="J7" s="2" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="3" t="s">
+    <row r="8" spans="1:10" ht="27.6">
+      <c r="A8" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="F8" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="G8" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="H8" s="3" t="s">
+      <c r="H8" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="I8" s="3" t="s">
+      <c r="I8" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="J8" s="3" t="s">
+      <c r="J8" s="2" t="s">
         <v>126</v>
       </c>
     </row>
@@ -5401,9 +5408,7 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>